<commit_message>
added html for iso 25059
</commit_message>
<xml_diff>
--- a/vocab_csv/spreadsheet.xlsx
+++ b/vocab_csv/spreadsheet.xlsx
@@ -71,7 +71,7 @@
     <t>dqv:Dimension</t>
   </si>
   <si>
-    <t>iso:ProductQuality</t>
+    <t>iso-25059:ProductQuality</t>
   </si>
   <si>
     <t>ISO/IEC 25010:2023, 3.1</t>
@@ -86,7 +86,7 @@
     <t>Capability of a product to provide a set of functions that covers all the specified tasks and intended users’ objectives.</t>
   </si>
   <si>
-    <t>iso:FunctionalSuitability</t>
+    <t>iso-25059:FunctionalSuitability</t>
   </si>
   <si>
     <t>ISO/IEC 25010:2023, 3.1.1</t>
@@ -150,7 +150,7 @@
     <t>Capability of a product to perform its specified function under specified conditions so that the response time and throughput rates meet the requirements</t>
   </si>
   <si>
-    <t xml:space="preserve">iso:PerformanceEfficiency
+    <t xml:space="preserve">iso-25059:PerformanceEfficiency
 </t>
   </si>
   <si>
@@ -211,7 +211,7 @@
     <t>Capability of a product to be recognized by users as appropriate for their needs</t>
   </si>
   <si>
-    <t>iso:InteractionCapability</t>
+    <t>iso-25059:InteractionCapability</t>
   </si>
   <si>
     <t>ISO/IEC 25010:2023, 3.4.1</t>
@@ -310,10 +310,10 @@
     <t>Degree to which appropriate information about the AI system is communicated to relevant stakeholders</t>
   </si>
   <si>
-    <t>iso:ProductQuality,iso:QualityInUse</t>
-  </si>
-  <si>
-    <t>iso:InteractionCapability,iso:Acceptability</t>
+    <t>iso-25059:ProductQuality,iso-25059:QualityInUse</t>
+  </si>
+  <si>
+    <t>iso-25059:InteractionCapability,iso-25059:Acceptability</t>
   </si>
   <si>
     <t xml:space="preserve">ISO/IEC 25059:2023, 3.1.5 , ISO/IEC DIS 25059:2025, 3.1.5 </t>
@@ -334,7 +334,7 @@
     <t>Capability of a product to perform specified functions without fault under normal operation</t>
   </si>
   <si>
-    <t xml:space="preserve">iso:Reliability
+    <t xml:space="preserve">iso-25059:Reliability
 </t>
   </si>
   <si>
@@ -396,7 +396,7 @@
     <t>Capability of a product to ensure that data are accessible only to those authorized to have access</t>
   </si>
   <si>
-    <t>iso:Security</t>
+    <t>iso-25059:Security</t>
   </si>
   <si>
     <t>ISO/IEC 25010:2023, 3.6.1</t>
@@ -471,7 +471,7 @@
     <t>Capability of a product to limit changes to one component from affecting other components</t>
   </si>
   <si>
-    <t>iso:Maintainability</t>
+    <t>iso-25059:Maintainability</t>
   </si>
   <si>
     <t>ISO/IEC 25010:2023, 3.7.1</t>
@@ -519,7 +519,7 @@
     <t>Capability of a product to enable an objective and feasible test to be designed and performed to determine whether a requirement is met</t>
   </si>
   <si>
-    <t>iso:Flexibility</t>
+    <t>iso-25059:Flexibility</t>
   </si>
   <si>
     <t>ISO/IEC 25010:2023, 3.7.5</t>
@@ -582,7 +582,7 @@
     <t>Capability of a product to constrain its operation to within safe parameters or states when encountering operational hazard</t>
   </si>
   <si>
-    <t>iso:Safety</t>
+    <t>iso-25059:Safety</t>
   </si>
   <si>
     <t>ISO/IEC 25010:2023, 3.9.1</t>
@@ -654,7 +654,7 @@
     <t>Capability of a product to perform its required functions efficiently while sharing a common environment and resources with other products, without detrimental impact on any other product</t>
   </si>
   <si>
-    <t xml:space="preserve">iso:Compatibility
+    <t xml:space="preserve">iso-25059:Compatibility
 </t>
   </si>
   <si>
@@ -683,7 +683,7 @@
     <t>Extent of benefit resulting from the use of a product, system or service</t>
   </si>
   <si>
-    <t>iso:QualityInUse</t>
+    <t>iso-25059:QualityInUse</t>
   </si>
   <si>
     <t>ISO/IEC 25019:2023,3.2.1</t>
@@ -695,7 +695,7 @@
     <t>Extent to which a system, product or service can be used by specified users  to achieve specified goals with effectiveness, efficiency, and satisfaction in a specified context of use</t>
   </si>
   <si>
-    <t>iso:Beneficialness</t>
+    <t>iso-25059:Beneficialness</t>
   </si>
   <si>
     <t>ISO/IEC 25019:2023,3.2.1.1</t>
@@ -737,7 +737,7 @@
     <t>Extent to which users or stakeholders accumulate knowledge or skill acquired over time, especially that gained in a particular profession</t>
   </si>
   <si>
-    <t>iso:Acceptability</t>
+    <t>iso-25059:Acceptability</t>
   </si>
   <si>
     <t>ISO/IEC 25019:2023,3.2.3.1</t>
@@ -779,7 +779,7 @@
     <t>Extent to which a product or system mitigates the potential risk to financial status, efficient operation, commercial property, reputation, or other aspects in the intended contexts of use</t>
   </si>
   <si>
-    <t>iso:RiskMitigation</t>
+    <t>iso-25059:RiskMitigation</t>
   </si>
   <si>
     <t>Definition of freedom from economic risk, ISO/IEC 25019:2023,3.2.2.1</t>
@@ -844,7 +844,7 @@
     <t>Degree to which an AI service meets stated and implied needs when used in a specified context of use</t>
   </si>
   <si>
-    <t>iso:AIServiceQuality</t>
+    <t>iso-25059:AIServiceQuality</t>
   </si>
   <si>
     <t>ISO/IEC TS 25011:2017, 3.2.1, IT service is replaced by AI service</t>
@@ -856,7 +856,7 @@
     <t>Degree to which an AI service supports all the specified goals, objectives and data specified by the user</t>
   </si>
   <si>
-    <t xml:space="preserve">iso:Suitability
+    <t xml:space="preserve">iso-25059:Suitability
 </t>
   </si>
   <si>
@@ -911,7 +911,7 @@
     <t>Degree to which users  can recognize whether an AI service is appropriate for their needs</t>
   </si>
   <si>
-    <t xml:space="preserve">iso:ServiceUsability
+    <t xml:space="preserve">iso-25059:ServiceUsability
 </t>
   </si>
   <si>
@@ -993,7 +993,7 @@
     <t>Degree to which an AI service ensures that data are accessible only to those authorized to have access</t>
   </si>
   <si>
-    <t>iso:ServiceSecurity</t>
+    <t>iso-25059:ServiceSecurity</t>
   </si>
   <si>
     <t>ISO/IEC TS 25011:2017, 3.2.3.1, IT service is replaced by AI service</t>
@@ -1008,7 +1008,7 @@
     <t>Degree to which an AI service prevents unauthorized access to or modification of data whether accidently or intentionally</t>
   </si>
   <si>
-    <t xml:space="preserve">iso:ServiceSecurity
+    <t xml:space="preserve">iso-25059:ServiceSecurity
 </t>
   </si>
   <si>
@@ -1042,7 +1042,7 @@
     <t>Degree to which the AI service is provided under all foreseeable circumstances, including mitigating the risks resulting from interruption to an acceptable level</t>
   </si>
   <si>
-    <t>iso:ServiceReliability</t>
+    <t>iso-25059:ServiceReliability</t>
   </si>
   <si>
     <t>ISO/IEC TS 25011:2017, 3.2.4.1, IT service is replaced by AI service</t>
@@ -1087,7 +1087,7 @@
     <t>Degree to which users have insight into the capabilities of the AI service, how they will be delivered, and progress toward their completion during delivery</t>
   </si>
   <si>
-    <t>iso:Tangibility</t>
+    <t>iso-25059:Tangibility</t>
   </si>
   <si>
     <t>ISO/IEC TS 25011:2017, 3.2.5.1, IT service is replaced by AI service</t>
@@ -1129,7 +1129,7 @@
     <t>Degree to which an AI service delivers outcomes within time limits</t>
   </si>
   <si>
-    <t>iso:Responsiveness</t>
+    <t>iso-25059:Responsiveness</t>
   </si>
   <si>
     <t>ISO/IEC TS 25011:2017, 3.2.6.1,  IT service is replaced by AI service</t>
@@ -1163,7 +1163,7 @@
     <t>Degree to which the AI service can be customized at the request of users</t>
   </si>
   <si>
-    <t>iso:ServiceAdaptability</t>
+    <t>iso-25059:ServiceAdaptability</t>
   </si>
   <si>
     <t>ISO/IEC DIS 25059:2025, 3.4.3</t>
@@ -1199,7 +1199,7 @@
     <t>Degree of effectiveness and efficiency with which an AI service can be analysed for deficiencies, gaps and failures</t>
   </si>
   <si>
-    <t>iso:ServiceMaintainability</t>
+    <t>iso-25059:ServiceMaintainability</t>
   </si>
   <si>
     <t>ISO/IEC TS 25011:2017, 3.2.8.1,  IT service is replaced by AI service</t>
@@ -23449,7 +23449,7 @@
       </c>
       <c r="F17" s="28"/>
       <c r="G17" s="11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H17" s="26" t="s">
         <v>619</v>
@@ -23573,7 +23573,7 @@
         <v>601</v>
       </c>
       <c r="G22" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H22" s="26" t="s">
         <v>637</v>
@@ -23597,7 +23597,7 @@
         <v>586</v>
       </c>
       <c r="G23" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H23" s="26" t="s">
         <v>637</v>

</xml_diff>

<commit_message>
add eu-aiact; make anonymous
</commit_message>
<xml_diff>
--- a/vocab_csv/spreadsheet.xlsx
+++ b/vocab_csv/spreadsheet.xlsx
@@ -1232,10 +1232,10 @@
     <t>Dimension</t>
   </si>
   <si>
-    <t>SystemQualityDimensions</t>
-  </si>
-  <si>
-    <t>System Quality Dimensions</t>
+    <t>SystemQuality</t>
+  </si>
+  <si>
+    <t>System Quality</t>
   </si>
   <si>
     <t>Quality associated with AI Systems</t>
@@ -1265,7 +1265,7 @@
     <t>AI Act Article 13</t>
   </si>
   <si>
-    <t>Interpretabilty</t>
+    <t>Interpretability</t>
   </si>
   <si>
     <t>Interpretabilty of system’s output</t>
@@ -1283,10 +1283,10 @@
     <t>AI Act Article 15(4)</t>
   </si>
   <si>
-    <t>ModelQualityDimensions</t>
-  </si>
-  <si>
-    <t>Model Quality Dimensions</t>
+    <t>ModelQuality</t>
+  </si>
+  <si>
+    <t>Model Quality</t>
   </si>
   <si>
     <t>Quality associated with AI Models</t>
@@ -1304,10 +1304,10 @@
     <t>AI Act Annex XIII (c)</t>
   </si>
   <si>
-    <t>DataQualityDimensions</t>
-  </si>
-  <si>
-    <t>Data Quality Dimensions</t>
+    <t>DataQuality</t>
+  </si>
+  <si>
+    <t>Data Quality</t>
   </si>
   <si>
     <t>Quality associated with data and data sets</t>

</xml_diff>